<commit_message>
pagamentos: planilha de hora extra com tipo de curso apos o nivel de docencia
- Modelo base_pagamento_extra.xlsx: Tipo de Curso passa a ficar logo apos
  o Nivel de Docencia, e entram os cabecalhos que faltavam (Tipo de Curso e
  Observacao), com o mesmo estilo dos demais e larguras de coluna proprias.
- _planilha_overtime grava os dados na nova ordem (tipo de curso na coluna 3,
  observacao na 10); a celula MES/ANO (D4) nao muda de lugar.
- Testes: posicoes de coluna revisadas e ordem completa dos 10 cabecalhos
  travada em teste novo.
</commit_message>
<xml_diff>
--- a/app/static/templates_excel/base_pagamento_extra.xlsx
+++ b/app/static/templates_excel/base_pagamento_extra.xlsx
@@ -1,167 +1,87 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joao.misturini\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8085"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8085" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Extra NEB" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extra NEB" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>CONTROLE DE PAGAMENTO EXTRACLASSE</t>
-  </si>
-  <si>
-    <t>UNIDADE EDUCACIONAL:</t>
-  </si>
-  <si>
-    <t>Faculdade Florianópolis</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MÊS/ANO:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t>Nome do Professor</t>
-  </si>
-  <si>
-    <t>Nível de Docência</t>
-  </si>
-  <si>
-    <t>Número de Horas</t>
-  </si>
-  <si>
-    <t>Valor H/a</t>
-  </si>
-  <si>
-    <t>Código Orçamentário</t>
-  </si>
-  <si>
-    <t>Justificativa</t>
-  </si>
-  <si>
-    <t>Assinatura do Coordenador Educacional</t>
-  </si>
-  <si>
-    <t>Assinatura do Diretor da Unidade Educacional</t>
-  </si>
-  <si>
-    <t>NES / NEB</t>
-  </si>
-  <si>
-    <t>Datas</t>
-  </si>
-  <si>
-    <t>Turno</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="16"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -212,70 +132,132 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="20">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -541,129 +523,169 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="36.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="29.140625" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" customWidth="1"/>
-    <col min="7" max="7" width="38.28515625" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col width="36.86" customWidth="1" min="1" max="1"/>
+    <col width="15.43" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16.57" customWidth="1" min="5" max="5"/>
+    <col width="29.14" customWidth="1" min="6" max="6"/>
+    <col width="19.14" customWidth="1" min="7" max="7"/>
+    <col width="38.29" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="14.86" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B2" s="18"/>
-      <c r="C2" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="14">
+    <row r="1">
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="21" customHeight="1">
+      <c r="B2" s="18" t="n"/>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>CONTROLE DE PAGAMENTO EXTRACLASSE</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+    </row>
+    <row r="3">
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>UNIDADE EDUCACIONAL:</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Faculdade Florianópolis</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MÊS/ANO: </t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="n">
         <v>45444</v>
       </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-    </row>
-    <row r="8" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="10"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="15"/>
-    </row>
-    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E25" s="15"/>
+      <c r="E4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="C5" s="1" t="n"/>
+      <c r="D5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="39.75" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Nome do Professor</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Nível de Docência</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Tipo de Curso</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Número de Horas</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Valor H/a</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Datas</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Turno</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Código Orçamentário</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Justificativa</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="16" t="n"/>
+      <c r="B7" s="17" t="n"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+    </row>
+    <row r="8" ht="18.75" customHeight="1">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="1" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Assinatura do Coordenador Educacional</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Assinatura do Diretor da Unidade Educacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>NES / NEB</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="n"/>
+    </row>
+    <row r="25">
+      <c r="E25" s="15" t="n"/>
     </row>
   </sheetData>
-  <sortState ref="A7:F18">
-    <sortCondition ref="A7"/>
-  </sortState>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup scale="69" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageSetup orientation="landscape" scale="69"/>
 </worksheet>
 </file>
</xml_diff>